<commit_message>
Rename bride-side tables to company and family names.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/2026-10-04-江林府喜宴-文華東方對照表.xlsx
+++ b/2026-10-04-江林府喜宴-文華東方對照表.xlsx
@@ -377,7 +377,7 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C4" s="0">
@@ -407,7 +407,7 @@
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C5" s="0">
@@ -437,7 +437,7 @@
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C6" s="0">
@@ -467,7 +467,7 @@
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C7" s="0">
@@ -497,7 +497,7 @@
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C8" s="0">
@@ -781,7 +781,7 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="6">
@@ -799,7 +799,7 @@
       </c>
       <c r="F2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="G2" s="9">
@@ -814,7 +814,7 @@
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="6">
@@ -832,7 +832,7 @@
       </c>
       <c r="F3" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="G3" s="9">
@@ -847,7 +847,7 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="6">
@@ -865,7 +865,7 @@
       </c>
       <c r="F4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="G4" s="9">
@@ -880,7 +880,7 @@
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="6">
@@ -898,7 +898,7 @@
       </c>
       <c r="F5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="G5" s="9">
@@ -913,7 +913,7 @@
       </c>
       <c r="B6" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="11">
@@ -944,7 +944,7 @@
       </c>
       <c r="B7" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="11">
@@ -975,7 +975,7 @@
       </c>
       <c r="B8" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="11">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="0">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="0">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="0">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="0">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="0">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="0">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="B16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="0">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="0">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="0">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C14" s="0">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C15" s="0">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="B16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C16" s="0">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C17" s="0">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C18" s="0">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B19" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C19" s="0">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C20" s="0">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="B21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C21" s="0">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C22" s="0">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="B23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C23" s="0">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="B24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C24" s="0">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森／萬里雲</t>
+          <t xml:space="preserve">艾克森科技／萬里雲科技</t>
         </is>
       </c>
       <c r="C25" s="0">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C26" s="0">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C27" s="0">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C28" s="0">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="B29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C29" s="0">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C30" s="0">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C31" s="0">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C32" s="0">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C33" s="0">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C34" s="0">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B35" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">艾克森</t>
+          <t xml:space="preserve">艾克森科技</t>
         </is>
       </c>
       <c r="C35" s="0">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B36" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C36" s="0">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C37" s="0">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B38" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C38" s="0">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B39" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C39" s="0">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="B40" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C40" s="0">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="B41" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C41" s="0">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B42" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C42" s="0">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B43" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C43" s="0">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B44" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C44" s="0">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B45" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C45" s="0">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="B46" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C46" s="0">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B47" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">創順</t>
+          <t xml:space="preserve">創順科技</t>
         </is>
       </c>
       <c r="C47" t="inlineStr" s="11">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="B48" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C48" s="0">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B49" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C49" s="0">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="B50" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C50" s="0">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="B51" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C51" s="0">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="B52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C52" s="0">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B53" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C53" s="0">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B54" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C54" s="0">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="B55" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C55" s="0">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="B56" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C56" s="0">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="B57" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C57" s="0">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="B58" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C58" s="0">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B59" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C59" s="0">
@@ -3163,7 +3163,7 @@
       </c>
       <c r="B60" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C60" s="0">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="B61" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C61" s="0">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="B62" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C62" s="0">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="B63" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C63" s="0">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B64" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C64" s="0">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="B65" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C65" s="0">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="B66" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C66" s="0">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B67" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方媽媽親戚</t>
+          <t xml:space="preserve">葉家親友</t>
         </is>
       </c>
       <c r="C67" s="0">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="B68" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C68" s="0">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B69" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C69" s="0">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B70" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C70" s="0">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="B71" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C71" s="0">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="B72" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C72" s="0">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="B73" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C73" s="0">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B74" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C74" s="0">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="B75" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C75" s="0">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="B76" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C76" s="0">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="B77" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C77" s="0">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="B78" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C78" s="0">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B79" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C79" s="0">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="B80" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C80" s="0">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B81" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C81" s="0">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="B82" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C82" s="0">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B83" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C83" s="0">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B84" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C84" s="0">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="B85" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C85" s="0">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="B86" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C86" s="0">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B87" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">仁寶</t>
+          <t xml:space="preserve">仁寶科技</t>
         </is>
       </c>
       <c r="C87" s="0">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B88" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C88" s="0">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="B89" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C89" s="0">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="B90" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C90" s="0">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B91" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C91" s="0">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B92" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C92" s="0">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="B93" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C93" s="0">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="B94" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C94" s="0">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="B95" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C95" s="0">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B96" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C96" s="0">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B97" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">女方爸爸親戚</t>
+          <t xml:space="preserve">林家親友</t>
         </is>
       </c>
       <c r="C97" s="0">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B108" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C108" s="0">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B109" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C109" s="0">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B110" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C110" s="0">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="B111" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C111" s="0">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B112" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C112" s="0">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="B113" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C113" s="0">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B114" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C114" s="0">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="B115" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C115" s="0">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="B116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C116" s="0">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B117" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">萬里雲</t>
+          <t xml:space="preserve">萬里雲科技</t>
         </is>
       </c>
       <c r="C117" s="0">
@@ -4443,7 +4443,7 @@
       </c>
       <c r="B118" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C118" s="0">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="B119" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C119" s="0">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="B120" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C120" s="0">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="B121" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C121" s="0">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B122" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C122" s="0">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="B123" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C123" s="0">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="B124" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C124" s="0">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="B125" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C125" s="0">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="B126" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C126" s="0">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B127" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C127" s="0">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="B128" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C128" s="0">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="B129" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C129" s="0">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="B130" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C130" s="0">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="B131" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C131" s="0">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="B132" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C132" s="0">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="B133" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C133" s="0">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="B134" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C134" s="0">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="B135" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C135" s="0">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="B136" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C136" s="0">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="B137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C137" s="0">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="B138" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C138" s="0">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="B139" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C139" t="inlineStr" s="11">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="B140" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C140" s="0">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B141" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C141" s="0">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="B142" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C142" s="0">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="B143" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C143" s="0">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B144" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C144" s="0">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="B145" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C145" s="0">
@@ -5069,7 +5069,7 @@
       </c>
       <c r="B146" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C146" s="0">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="B147" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C147" s="0">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="B148" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C148" s="0">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="B149" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C149" s="0">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B150" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">新郎好友</t>
+          <t xml:space="preserve">伊諾科技</t>
         </is>
       </c>
       <c r="C150" t="inlineStr" s="11">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="B151" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C151" s="0">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="B152" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C152" s="0">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="B153" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C153" s="0">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B154" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C154" s="0">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="B155" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C155" s="0">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="B156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C156" s="0">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B157" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C157" s="0">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="B158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C158" s="0">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="B159" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C159" s="0">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="B160" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">男方親友</t>
+          <t xml:space="preserve">江家親友</t>
         </is>
       </c>
       <c r="C160" s="0">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="B161" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C161" s="0">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B162" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C162" s="0">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="B163" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C163" s="0">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="B164" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C164" s="0">
@@ -5501,7 +5501,7 @@
       </c>
       <c r="B165" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C165" s="0">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="B166" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C166" s="0">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="B167" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C167" s="0">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="B168" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C168" s="0">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="B169" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C169" s="0">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="B170" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C170" s="0">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="B171" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C171" s="0">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="B172" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C172" s="0">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="B173" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C173" s="0">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="B174" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C174" s="0">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="B175" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C175" s="0">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="B176" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C176" s="0">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="B177" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C177" s="0">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="B178" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C178" s="0">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="B179" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C179" s="0">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B180" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C180" s="0">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="B181" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C181" s="0">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="B192" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C192" s="0">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B193" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C193" s="0">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="B194" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C194" s="0">
@@ -6189,7 +6189,7 @@
       </c>
       <c r="B195" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C195" s="0">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="B196" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C196" s="0">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="B197" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C197" s="0">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="B198" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C198" s="0">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="B199" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C199" s="0">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="B200" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C200" s="0">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="B201" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">爸爸同學</t>
+          <t xml:space="preserve">新郎父親好友</t>
         </is>
       </c>
       <c r="C201" s="0">

</xml_diff>